<commit_message>
Plantilla de gravedad específica (arcillas): versión actualizada con las firmas
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/GDA-FLC-006_gravedad_arcilla.xlsx
+++ b/templates/GDA-FLC-006_gravedad_arcilla.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GeoDelta Líneas\Dropbox\14. GEODELTA\014 FORMATOS ACTUALIZADOS 2026\FORMATOS PARA DIGITAR ACTUALIZADOS 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DCM-04\Dropbox\14. GEODELTA\014 FORMATOS ACTUALIZADOS 2026\FORMATOS PARA DIGITAR ACTUALIZADOS 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8911D77-09F8-4AED-8446-396FE504CD80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F58A1CD9-CF91-4421-859A-56FF59D5E168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$A$1:$K$43</definedName>
     <definedName name="GFDGSD">[1]L!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2030,19 +2030,145 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="72" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="80" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="81" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2055,11 +2181,9 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2067,141 +2191,17 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="80" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="81" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="72" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2487,6 +2487,93 @@
     </xdr:pic>
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>619125</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1110192</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>265194</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Imagen 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B219896C-77CF-42CE-A4FE-B4EF9AB7A3D7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:srcRect l="88188"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7941469" y="8751094"/>
+          <a:ext cx="1776942" cy="693819"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>428625</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>288395</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>119913</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Imagen 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F2D8DCB3-4F4B-4BA0-9E8F-795371300FDE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11477625" y="8703469"/>
+          <a:ext cx="1550458" cy="905725"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2745,21 +2832,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:46" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="133"/>
-      <c r="B1" s="134"/>
-      <c r="C1" s="139" t="s">
+      <c r="A1" s="194"/>
+      <c r="B1" s="195"/>
+      <c r="C1" s="196" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="140"/>
-      <c r="E1" s="140"/>
-      <c r="F1" s="140"/>
-      <c r="G1" s="140"/>
-      <c r="H1" s="134"/>
-      <c r="I1" s="141" t="s">
+      <c r="D1" s="197"/>
+      <c r="E1" s="197"/>
+      <c r="F1" s="197"/>
+      <c r="G1" s="197"/>
+      <c r="H1" s="195"/>
+      <c r="I1" s="198" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="142"/>
-      <c r="K1" s="143"/>
+      <c r="J1" s="199"/>
+      <c r="K1" s="200"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
       <c r="N1" s="2"/>
@@ -2789,31 +2876,31 @@
       <c r="AL1" s="3"/>
       <c r="AM1" s="3"/>
       <c r="AN1" s="3"/>
-      <c r="AO1" s="159" t="s">
+      <c r="AO1" s="186" t="s">
         <v>2</v>
       </c>
-      <c r="AP1" s="160"/>
-      <c r="AQ1" s="160"/>
+      <c r="AP1" s="143"/>
+      <c r="AQ1" s="143"/>
       <c r="AR1" s="3"/>
       <c r="AS1" s="3"/>
       <c r="AT1" s="3"/>
     </row>
     <row r="2" spans="1:46" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="135"/>
-      <c r="B2" s="136"/>
-      <c r="C2" s="161" t="s">
+      <c r="A2" s="188"/>
+      <c r="B2" s="141"/>
+      <c r="C2" s="187" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="131"/>
-      <c r="E2" s="131"/>
-      <c r="F2" s="131"/>
-      <c r="G2" s="131"/>
-      <c r="H2" s="132"/>
-      <c r="I2" s="163" t="s">
+      <c r="D2" s="140"/>
+      <c r="E2" s="140"/>
+      <c r="F2" s="140"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="138"/>
+      <c r="I2" s="190" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="153"/>
-      <c r="K2" s="154"/>
+      <c r="J2" s="151"/>
+      <c r="K2" s="182"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
       <c r="N2" s="2"/>
@@ -2851,19 +2938,19 @@
       <c r="AT2" s="3"/>
     </row>
     <row r="3" spans="1:46" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="135"/>
-      <c r="B3" s="136"/>
-      <c r="C3" s="135"/>
-      <c r="D3" s="131"/>
-      <c r="E3" s="131"/>
-      <c r="F3" s="131"/>
-      <c r="G3" s="131"/>
-      <c r="H3" s="132"/>
-      <c r="I3" s="163" t="s">
+      <c r="A3" s="188"/>
+      <c r="B3" s="141"/>
+      <c r="C3" s="188"/>
+      <c r="D3" s="140"/>
+      <c r="E3" s="140"/>
+      <c r="F3" s="140"/>
+      <c r="G3" s="140"/>
+      <c r="H3" s="138"/>
+      <c r="I3" s="190" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="153"/>
-      <c r="K3" s="154"/>
+      <c r="J3" s="151"/>
+      <c r="K3" s="182"/>
       <c r="L3" s="1"/>
       <c r="M3" s="5" t="s">
         <v>6</v>
@@ -2887,12 +2974,12 @@
       <c r="AD3" s="3"/>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
-      <c r="AG3" s="164" t="s">
+      <c r="AG3" s="191" t="s">
         <v>6</v>
       </c>
-      <c r="AH3" s="160"/>
-      <c r="AI3" s="160"/>
-      <c r="AJ3" s="160"/>
+      <c r="AH3" s="143"/>
+      <c r="AI3" s="143"/>
+      <c r="AJ3" s="143"/>
       <c r="AK3" s="3"/>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -2911,19 +2998,19 @@
       <c r="AT3" s="3"/>
     </row>
     <row r="4" spans="1:46" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="137"/>
-      <c r="B4" s="138"/>
-      <c r="C4" s="137"/>
-      <c r="D4" s="162"/>
-      <c r="E4" s="162"/>
-      <c r="F4" s="162"/>
-      <c r="G4" s="162"/>
-      <c r="H4" s="138"/>
-      <c r="I4" s="166" t="s">
+      <c r="A4" s="189"/>
+      <c r="B4" s="146"/>
+      <c r="C4" s="189"/>
+      <c r="D4" s="145"/>
+      <c r="E4" s="145"/>
+      <c r="F4" s="145"/>
+      <c r="G4" s="145"/>
+      <c r="H4" s="146"/>
+      <c r="I4" s="193" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="162"/>
-      <c r="K4" s="138"/>
+      <c r="J4" s="145"/>
+      <c r="K4" s="146"/>
       <c r="L4" s="1"/>
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
@@ -2945,10 +3032,10 @@
       <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
       <c r="AF4" s="3"/>
-      <c r="AG4" s="160"/>
-      <c r="AH4" s="160"/>
-      <c r="AI4" s="160"/>
-      <c r="AJ4" s="160"/>
+      <c r="AG4" s="143"/>
+      <c r="AH4" s="143"/>
+      <c r="AI4" s="143"/>
+      <c r="AJ4" s="143"/>
       <c r="AK4" s="3"/>
       <c r="AL4" s="3"/>
       <c r="AM4" s="3"/>
@@ -2968,15 +3055,15 @@
     </row>
     <row r="5" spans="1:46" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="98"/>
-      <c r="B5" s="165"/>
-      <c r="C5" s="131"/>
-      <c r="D5" s="131"/>
-      <c r="E5" s="131"/>
-      <c r="F5" s="131"/>
-      <c r="G5" s="131"/>
-      <c r="H5" s="131"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="131"/>
+      <c r="B5" s="192"/>
+      <c r="C5" s="140"/>
+      <c r="D5" s="140"/>
+      <c r="E5" s="140"/>
+      <c r="F5" s="140"/>
+      <c r="G5" s="140"/>
+      <c r="H5" s="140"/>
+      <c r="I5" s="140"/>
+      <c r="J5" s="140"/>
       <c r="K5" s="99"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -2999,10 +3086,10 @@
       <c r="AD5" s="3"/>
       <c r="AE5" s="3"/>
       <c r="AF5" s="3"/>
-      <c r="AG5" s="160"/>
-      <c r="AH5" s="160"/>
-      <c r="AI5" s="160"/>
-      <c r="AJ5" s="160"/>
+      <c r="AG5" s="143"/>
+      <c r="AH5" s="143"/>
+      <c r="AI5" s="143"/>
+      <c r="AJ5" s="143"/>
       <c r="AK5" s="3"/>
       <c r="AL5" s="3"/>
       <c r="AM5" s="3"/>
@@ -3025,17 +3112,17 @@
       <c r="B6" s="101" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="144"/>
-      <c r="D6" s="145"/>
-      <c r="E6" s="145"/>
-      <c r="F6" s="145"/>
-      <c r="G6" s="146" t="s">
+      <c r="C6" s="201"/>
+      <c r="D6" s="173"/>
+      <c r="E6" s="173"/>
+      <c r="F6" s="173"/>
+      <c r="G6" s="202" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="147"/>
-      <c r="I6" s="148"/>
-      <c r="J6" s="145"/>
-      <c r="K6" s="149"/>
+      <c r="H6" s="162"/>
+      <c r="I6" s="203"/>
+      <c r="J6" s="173"/>
+      <c r="K6" s="204"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
       <c r="N6" s="11" t="s">
@@ -3091,17 +3178,17 @@
       <c r="B7" s="102" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="157"/>
-      <c r="D7" s="153"/>
-      <c r="E7" s="153"/>
-      <c r="F7" s="153"/>
-      <c r="G7" s="150" t="s">
+      <c r="C7" s="183"/>
+      <c r="D7" s="151"/>
+      <c r="E7" s="151"/>
+      <c r="F7" s="151"/>
+      <c r="G7" s="205" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="151"/>
-      <c r="I7" s="152"/>
-      <c r="J7" s="153"/>
-      <c r="K7" s="154"/>
+      <c r="H7" s="137"/>
+      <c r="I7" s="181"/>
+      <c r="J7" s="151"/>
+      <c r="K7" s="182"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
       <c r="N7" s="11" t="s">
@@ -3153,17 +3240,17 @@
       <c r="B8" s="102" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="157"/>
-      <c r="D8" s="153"/>
-      <c r="E8" s="153"/>
-      <c r="F8" s="153"/>
-      <c r="G8" s="150" t="s">
+      <c r="C8" s="183"/>
+      <c r="D8" s="151"/>
+      <c r="E8" s="151"/>
+      <c r="F8" s="151"/>
+      <c r="G8" s="205" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="151"/>
-      <c r="I8" s="152"/>
-      <c r="J8" s="153"/>
-      <c r="K8" s="154"/>
+      <c r="H8" s="137"/>
+      <c r="I8" s="181"/>
+      <c r="J8" s="151"/>
+      <c r="K8" s="182"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1">
         <f>17-2.57</f>
@@ -3220,14 +3307,14 @@
       <c r="B9" s="102" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="157"/>
-      <c r="D9" s="153"/>
-      <c r="E9" s="153"/>
-      <c r="F9" s="153"/>
-      <c r="G9" s="150" t="s">
+      <c r="C9" s="183"/>
+      <c r="D9" s="151"/>
+      <c r="E9" s="151"/>
+      <c r="F9" s="151"/>
+      <c r="G9" s="205" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="151"/>
+      <c r="H9" s="137"/>
       <c r="I9" s="103" t="s">
         <v>22</v>
       </c>
@@ -3286,20 +3373,20 @@
       <c r="B10" s="105" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="157"/>
-      <c r="D10" s="153"/>
-      <c r="E10" s="153"/>
-      <c r="F10" s="153"/>
-      <c r="G10" s="155" t="s">
+      <c r="C10" s="183"/>
+      <c r="D10" s="151"/>
+      <c r="E10" s="151"/>
+      <c r="F10" s="151"/>
+      <c r="G10" s="206" t="s">
         <v>25</v>
       </c>
-      <c r="H10" s="156"/>
-      <c r="I10" s="157" t="str">
+      <c r="H10" s="207"/>
+      <c r="I10" s="183" t="str">
         <f>CONCATENATE(J9,," ",K9,"-",D12,"-",B45,F12)</f>
         <v xml:space="preserve"> --</v>
       </c>
-      <c r="J10" s="153"/>
-      <c r="K10" s="154"/>
+      <c r="J10" s="151"/>
+      <c r="K10" s="182"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="11" t="s">
@@ -3348,15 +3435,15 @@
     </row>
     <row r="11" spans="1:46" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="106"/>
-      <c r="B11" s="167"/>
-      <c r="C11" s="168"/>
-      <c r="D11" s="168"/>
-      <c r="E11" s="168"/>
-      <c r="F11" s="168"/>
-      <c r="G11" s="168"/>
-      <c r="H11" s="168"/>
-      <c r="I11" s="168"/>
-      <c r="J11" s="168"/>
+      <c r="B11" s="184"/>
+      <c r="C11" s="179"/>
+      <c r="D11" s="179"/>
+      <c r="E11" s="179"/>
+      <c r="F11" s="179"/>
+      <c r="G11" s="179"/>
+      <c r="H11" s="179"/>
+      <c r="I11" s="179"/>
+      <c r="J11" s="179"/>
       <c r="K11" s="107"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
@@ -3413,10 +3500,10 @@
         <v>28</v>
       </c>
       <c r="F12" s="17"/>
-      <c r="G12" s="158" t="s">
+      <c r="G12" s="208" t="s">
         <v>29</v>
       </c>
-      <c r="H12" s="147"/>
+      <c r="H12" s="162"/>
       <c r="I12" s="18"/>
       <c r="J12" s="19" t="s">
         <v>30</v>
@@ -3469,15 +3556,15 @@
       <c r="B13" s="102" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="169"/>
-      <c r="D13" s="153"/>
-      <c r="E13" s="153"/>
-      <c r="F13" s="153"/>
-      <c r="G13" s="153"/>
-      <c r="H13" s="153"/>
-      <c r="I13" s="153"/>
-      <c r="J13" s="153"/>
-      <c r="K13" s="154"/>
+      <c r="C13" s="185"/>
+      <c r="D13" s="151"/>
+      <c r="E13" s="151"/>
+      <c r="F13" s="151"/>
+      <c r="G13" s="151"/>
+      <c r="H13" s="151"/>
+      <c r="I13" s="151"/>
+      <c r="J13" s="151"/>
+      <c r="K13" s="182"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="11"/>
@@ -3629,19 +3716,19 @@
       <c r="AT15" s="3"/>
     </row>
     <row r="16" spans="1:46" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="170" t="s">
+      <c r="A16" s="169" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="171"/>
-      <c r="C16" s="171"/>
-      <c r="D16" s="171"/>
-      <c r="E16" s="171"/>
-      <c r="F16" s="171"/>
-      <c r="G16" s="171"/>
-      <c r="H16" s="171"/>
-      <c r="I16" s="171"/>
-      <c r="J16" s="171"/>
-      <c r="K16" s="172"/>
+      <c r="B16" s="170"/>
+      <c r="C16" s="170"/>
+      <c r="D16" s="170"/>
+      <c r="E16" s="170"/>
+      <c r="F16" s="170"/>
+      <c r="G16" s="170"/>
+      <c r="H16" s="170"/>
+      <c r="I16" s="170"/>
+      <c r="J16" s="170"/>
+      <c r="K16" s="171"/>
       <c r="L16" s="20"/>
       <c r="M16" s="20"/>
       <c r="N16" s="20"/>
@@ -3741,12 +3828,12 @@
     <row r="18" spans="1:46" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="113"/>
       <c r="B18" s="114"/>
-      <c r="C18" s="173" t="s">
+      <c r="C18" s="161" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="147"/>
-      <c r="E18" s="147"/>
-      <c r="F18" s="174"/>
+      <c r="D18" s="162"/>
+      <c r="E18" s="162"/>
+      <c r="F18" s="163"/>
       <c r="G18" s="22">
         <v>1</v>
       </c>
@@ -3757,19 +3844,19 @@
       <c r="L18" s="20"/>
       <c r="M18" s="20"/>
       <c r="N18" s="20"/>
-      <c r="O18" s="202" t="s">
+      <c r="O18" s="133" t="s">
         <v>91</v>
       </c>
-      <c r="P18" s="202"/>
-      <c r="Q18" s="202"/>
-      <c r="R18" s="202"/>
-      <c r="S18" s="202"/>
-      <c r="T18" s="202"/>
-      <c r="U18" s="202"/>
-      <c r="V18" s="202"/>
-      <c r="W18" s="202"/>
-      <c r="X18" s="202"/>
-      <c r="Y18" s="202"/>
+      <c r="P18" s="133"/>
+      <c r="Q18" s="133"/>
+      <c r="R18" s="133"/>
+      <c r="S18" s="133"/>
+      <c r="T18" s="133"/>
+      <c r="U18" s="133"/>
+      <c r="V18" s="133"/>
+      <c r="W18" s="133"/>
+      <c r="X18" s="133"/>
+      <c r="Y18" s="133"/>
       <c r="Z18" s="21"/>
       <c r="AA18" s="21"/>
       <c r="AB18" s="21"/>
@@ -3801,11 +3888,11 @@
     <row r="19" spans="1:46" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="113"/>
       <c r="B19" s="114"/>
-      <c r="C19" s="175" t="s">
+      <c r="C19" s="172" t="s">
         <v>35</v>
       </c>
-      <c r="D19" s="145"/>
-      <c r="E19" s="176"/>
+      <c r="D19" s="173"/>
+      <c r="E19" s="166"/>
       <c r="F19" s="26" t="s">
         <v>36</v>
       </c>
@@ -3817,17 +3904,17 @@
       <c r="L19" s="20"/>
       <c r="M19" s="20"/>
       <c r="N19" s="20"/>
-      <c r="O19" s="202"/>
-      <c r="P19" s="202"/>
-      <c r="Q19" s="202"/>
-      <c r="R19" s="202"/>
-      <c r="S19" s="202"/>
-      <c r="T19" s="202"/>
-      <c r="U19" s="202"/>
-      <c r="V19" s="202"/>
-      <c r="W19" s="202"/>
-      <c r="X19" s="202"/>
-      <c r="Y19" s="202"/>
+      <c r="O19" s="133"/>
+      <c r="P19" s="133"/>
+      <c r="Q19" s="133"/>
+      <c r="R19" s="133"/>
+      <c r="S19" s="133"/>
+      <c r="T19" s="133"/>
+      <c r="U19" s="133"/>
+      <c r="V19" s="133"/>
+      <c r="W19" s="133"/>
+      <c r="X19" s="133"/>
+      <c r="Y19" s="133"/>
       <c r="Z19" s="21"/>
       <c r="AA19" s="21"/>
       <c r="AB19" s="21"/>
@@ -3859,11 +3946,11 @@
     <row r="20" spans="1:46" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="113"/>
       <c r="B20" s="114"/>
-      <c r="C20" s="186" t="s">
+      <c r="C20" s="150" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="153"/>
-      <c r="E20" s="187"/>
+      <c r="D20" s="151"/>
+      <c r="E20" s="152"/>
       <c r="F20" s="30" t="s">
         <v>38</v>
       </c>
@@ -3875,25 +3962,25 @@
       <c r="L20" s="20"/>
       <c r="M20" s="20"/>
       <c r="N20" s="20"/>
-      <c r="O20" s="203" t="s">
+      <c r="O20" s="134" t="s">
         <v>87</v>
       </c>
-      <c r="P20" s="203"/>
+      <c r="P20" s="134"/>
       <c r="Q20" s="127"/>
-      <c r="R20" s="204" t="s">
+      <c r="R20" s="135" t="s">
         <v>88</v>
       </c>
-      <c r="S20" s="204"/>
+      <c r="S20" s="135"/>
       <c r="T20" s="127"/>
-      <c r="U20" s="204" t="s">
+      <c r="U20" s="135" t="s">
         <v>89</v>
       </c>
-      <c r="V20" s="204"/>
+      <c r="V20" s="135"/>
       <c r="W20" s="127"/>
-      <c r="X20" s="204" t="s">
+      <c r="X20" s="135" t="s">
         <v>90</v>
       </c>
-      <c r="Y20" s="204"/>
+      <c r="Y20" s="135"/>
       <c r="Z20" s="21"/>
       <c r="AA20" s="21"/>
       <c r="AB20" s="21"/>
@@ -3925,11 +4012,11 @@
     <row r="21" spans="1:46" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="113"/>
       <c r="B21" s="114"/>
-      <c r="C21" s="186" t="s">
+      <c r="C21" s="150" t="s">
         <v>40</v>
       </c>
-      <c r="D21" s="153"/>
-      <c r="E21" s="187"/>
+      <c r="D21" s="151"/>
+      <c r="E21" s="152"/>
       <c r="F21" s="30" t="s">
         <v>38</v>
       </c>
@@ -4002,11 +4089,11 @@
     <row r="22" spans="1:46" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="113"/>
       <c r="B22" s="114"/>
-      <c r="C22" s="186" t="s">
+      <c r="C22" s="150" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="153"/>
-      <c r="E22" s="187"/>
+      <c r="D22" s="151"/>
+      <c r="E22" s="152"/>
       <c r="F22" s="30" t="s">
         <v>38</v>
       </c>
@@ -4076,11 +4163,11 @@
     <row r="23" spans="1:46" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="113"/>
       <c r="B23" s="114"/>
-      <c r="C23" s="186" t="s">
+      <c r="C23" s="150" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="153"/>
-      <c r="E23" s="187"/>
+      <c r="D23" s="151"/>
+      <c r="E23" s="152"/>
       <c r="F23" s="30" t="s">
         <v>44</v>
       </c>
@@ -4150,11 +4237,11 @@
     <row r="24" spans="1:46" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="113"/>
       <c r="B24" s="114"/>
-      <c r="C24" s="186" t="s">
+      <c r="C24" s="150" t="s">
         <v>45</v>
       </c>
-      <c r="D24" s="153"/>
-      <c r="E24" s="187"/>
+      <c r="D24" s="151"/>
+      <c r="E24" s="152"/>
       <c r="F24" s="30" t="s">
         <v>46</v>
       </c>
@@ -4227,11 +4314,11 @@
     <row r="25" spans="1:46" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="113"/>
       <c r="B25" s="114"/>
-      <c r="C25" s="189" t="s">
+      <c r="C25" s="154" t="s">
         <v>47</v>
       </c>
-      <c r="D25" s="182"/>
-      <c r="E25" s="178"/>
+      <c r="D25" s="155"/>
+      <c r="E25" s="156"/>
       <c r="F25" s="129" t="s">
         <v>46</v>
       </c>
@@ -4304,12 +4391,12 @@
     <row r="26" spans="1:46" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="113"/>
       <c r="B26" s="114"/>
-      <c r="C26" s="190" t="s">
+      <c r="C26" s="157" t="s">
         <v>48</v>
       </c>
-      <c r="D26" s="191"/>
-      <c r="E26" s="191"/>
-      <c r="F26" s="192"/>
+      <c r="D26" s="158"/>
+      <c r="E26" s="158"/>
+      <c r="F26" s="159"/>
       <c r="G26" s="128" t="e">
         <f>IF(D32&gt;0.1,F49,IF(D32=0,F50))</f>
         <v>#VALUE!</v>
@@ -4379,8 +4466,8 @@
     <row r="27" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="113"/>
       <c r="B27" s="114"/>
-      <c r="C27" s="193"/>
-      <c r="D27" s="131"/>
+      <c r="C27" s="160"/>
+      <c r="D27" s="140"/>
       <c r="E27" s="114"/>
       <c r="F27" s="114"/>
       <c r="G27" s="117"/>
@@ -4581,13 +4668,13 @@
     <row r="30" spans="1:46" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="113"/>
       <c r="B30" s="114"/>
-      <c r="C30" s="173" t="s">
+      <c r="C30" s="161" t="s">
         <v>49</v>
       </c>
-      <c r="D30" s="147"/>
-      <c r="E30" s="147"/>
-      <c r="F30" s="147"/>
-      <c r="G30" s="174"/>
+      <c r="D30" s="162"/>
+      <c r="E30" s="162"/>
+      <c r="F30" s="162"/>
+      <c r="G30" s="163"/>
       <c r="H30" s="114"/>
       <c r="I30" s="114"/>
       <c r="J30" s="116"/>
@@ -4648,14 +4735,14 @@
       <c r="C31" s="45" t="s">
         <v>50</v>
       </c>
-      <c r="D31" s="194" t="s">
+      <c r="D31" s="164" t="s">
         <v>51</v>
       </c>
-      <c r="E31" s="176"/>
-      <c r="F31" s="194" t="s">
+      <c r="E31" s="166"/>
+      <c r="F31" s="164" t="s">
         <v>52</v>
       </c>
-      <c r="G31" s="195"/>
+      <c r="G31" s="165"/>
       <c r="H31" s="114"/>
       <c r="I31" s="114"/>
       <c r="J31" s="114"/>
@@ -4714,13 +4801,13 @@
       <c r="A32" s="113"/>
       <c r="B32" s="114"/>
       <c r="C32" s="47"/>
-      <c r="D32" s="196"/>
-      <c r="E32" s="178"/>
-      <c r="F32" s="196">
+      <c r="D32" s="167"/>
+      <c r="E32" s="156"/>
+      <c r="F32" s="167">
         <f>100-D32</f>
         <v>100</v>
       </c>
-      <c r="G32" s="183"/>
+      <c r="G32" s="168"/>
       <c r="H32" s="114"/>
       <c r="I32" s="114"/>
       <c r="J32" s="114"/>
@@ -4778,13 +4865,13 @@
     <row r="33" spans="1:46" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="113"/>
       <c r="B33" s="119"/>
-      <c r="C33" s="177" t="s">
+      <c r="C33" s="174" t="s">
         <v>53</v>
       </c>
-      <c r="D33" s="178"/>
-      <c r="E33" s="181"/>
-      <c r="F33" s="182"/>
-      <c r="G33" s="183"/>
+      <c r="D33" s="156"/>
+      <c r="E33" s="177"/>
+      <c r="F33" s="155"/>
+      <c r="G33" s="168"/>
       <c r="H33" s="114"/>
       <c r="I33" s="114"/>
       <c r="J33" s="114"/>
@@ -4842,11 +4929,11 @@
     <row r="34" spans="1:46" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="113"/>
       <c r="B34" s="114"/>
-      <c r="C34" s="179"/>
-      <c r="D34" s="180"/>
-      <c r="E34" s="184"/>
-      <c r="F34" s="168"/>
-      <c r="G34" s="185"/>
+      <c r="C34" s="175"/>
+      <c r="D34" s="176"/>
+      <c r="E34" s="178"/>
+      <c r="F34" s="179"/>
+      <c r="G34" s="180"/>
       <c r="H34" s="114"/>
       <c r="I34" s="114"/>
       <c r="J34" s="114"/>
@@ -4962,23 +5049,23 @@
       <c r="AT35" s="13"/>
     </row>
     <row r="36" spans="1:46" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="188" t="s">
+      <c r="A36" s="153" t="s">
         <v>57</v>
       </c>
-      <c r="B36" s="131"/>
-      <c r="C36" s="131"/>
-      <c r="D36" s="131"/>
-      <c r="E36" s="131"/>
-      <c r="F36" s="130" t="s">
+      <c r="B36" s="140"/>
+      <c r="C36" s="140"/>
+      <c r="D36" s="140"/>
+      <c r="E36" s="140"/>
+      <c r="F36" s="139" t="s">
         <v>58</v>
       </c>
-      <c r="G36" s="131"/>
+      <c r="G36" s="140"/>
       <c r="H36" s="121"/>
-      <c r="I36" s="130" t="s">
+      <c r="I36" s="139" t="s">
         <v>59</v>
       </c>
-      <c r="J36" s="131"/>
-      <c r="K36" s="132"/>
+      <c r="J36" s="140"/>
+      <c r="K36" s="138"/>
       <c r="L36" s="3"/>
       <c r="O36" s="127">
         <v>20.000000000000021</v>
@@ -5028,13 +5115,13 @@
       <c r="AT36" s="13"/>
     </row>
     <row r="37" spans="1:46" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="200" t="s">
+      <c r="A37" s="148" t="s">
         <v>60</v>
       </c>
-      <c r="B37" s="131"/>
-      <c r="C37" s="131"/>
-      <c r="D37" s="131"/>
-      <c r="E37" s="131"/>
+      <c r="B37" s="140"/>
+      <c r="C37" s="140"/>
+      <c r="D37" s="140"/>
+      <c r="E37" s="140"/>
       <c r="F37" s="123"/>
       <c r="G37" s="124"/>
       <c r="H37" s="121"/>
@@ -5090,11 +5177,11 @@
       <c r="AT37" s="13"/>
     </row>
     <row r="38" spans="1:46" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="201"/>
-      <c r="B38" s="131"/>
-      <c r="C38" s="131"/>
-      <c r="D38" s="131"/>
-      <c r="E38" s="131"/>
+      <c r="A38" s="149"/>
+      <c r="B38" s="140"/>
+      <c r="C38" s="140"/>
+      <c r="D38" s="140"/>
+      <c r="E38" s="140"/>
       <c r="F38" s="125"/>
       <c r="G38" s="121"/>
       <c r="H38" s="121"/>
@@ -5150,11 +5237,11 @@
       <c r="AT38" s="13"/>
     </row>
     <row r="39" spans="1:46" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="201"/>
-      <c r="B39" s="131"/>
-      <c r="C39" s="131"/>
-      <c r="D39" s="131"/>
-      <c r="E39" s="131"/>
+      <c r="A39" s="149"/>
+      <c r="B39" s="140"/>
+      <c r="C39" s="140"/>
+      <c r="D39" s="140"/>
+      <c r="E39" s="140"/>
       <c r="F39" s="125"/>
       <c r="G39" s="121"/>
       <c r="H39" s="121"/>
@@ -5210,17 +5297,17 @@
       <c r="AT39" s="21"/>
     </row>
     <row r="40" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="201"/>
-      <c r="B40" s="131"/>
-      <c r="C40" s="131"/>
-      <c r="D40" s="131"/>
-      <c r="E40" s="131"/>
-      <c r="F40" s="208"/>
-      <c r="G40" s="209"/>
+      <c r="A40" s="149"/>
+      <c r="B40" s="140"/>
+      <c r="C40" s="140"/>
+      <c r="D40" s="140"/>
+      <c r="E40" s="140"/>
+      <c r="F40" s="130"/>
+      <c r="G40" s="131"/>
       <c r="H40" s="126"/>
-      <c r="I40" s="208"/>
-      <c r="J40" s="209"/>
-      <c r="K40" s="210"/>
+      <c r="I40" s="130"/>
+      <c r="J40" s="131"/>
+      <c r="K40" s="132"/>
       <c r="L40" s="3"/>
       <c r="O40" s="127">
         <v>20.400000000000027</v>
@@ -5270,21 +5357,21 @@
       <c r="AT40" s="13"/>
     </row>
     <row r="41" spans="1:46" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="201"/>
-      <c r="B41" s="131"/>
-      <c r="C41" s="131"/>
-      <c r="D41" s="131"/>
-      <c r="E41" s="131"/>
-      <c r="F41" s="207" t="s">
+      <c r="A41" s="149"/>
+      <c r="B41" s="140"/>
+      <c r="C41" s="140"/>
+      <c r="D41" s="140"/>
+      <c r="E41" s="140"/>
+      <c r="F41" s="136" t="s">
         <v>63</v>
       </c>
-      <c r="G41" s="151"/>
+      <c r="G41" s="137"/>
       <c r="H41" s="126"/>
-      <c r="I41" s="207" t="s">
+      <c r="I41" s="136" t="s">
         <v>86</v>
       </c>
-      <c r="J41" s="151"/>
-      <c r="K41" s="132"/>
+      <c r="J41" s="137"/>
+      <c r="K41" s="138"/>
       <c r="L41" s="49"/>
       <c r="O41" s="127">
         <v>20.500000000000028</v>
@@ -5334,21 +5421,21 @@
       <c r="AT41" s="21"/>
     </row>
     <row r="42" spans="1:46" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="201"/>
-      <c r="B42" s="131"/>
-      <c r="C42" s="131"/>
-      <c r="D42" s="131"/>
-      <c r="E42" s="131"/>
-      <c r="F42" s="130" t="s">
+      <c r="A42" s="149"/>
+      <c r="B42" s="140"/>
+      <c r="C42" s="140"/>
+      <c r="D42" s="140"/>
+      <c r="E42" s="140"/>
+      <c r="F42" s="139" t="s">
         <v>65</v>
       </c>
-      <c r="G42" s="131"/>
+      <c r="G42" s="140"/>
       <c r="H42" s="121"/>
-      <c r="I42" s="130" t="s">
+      <c r="I42" s="139" t="s">
         <v>66</v>
       </c>
-      <c r="J42" s="131"/>
-      <c r="K42" s="136"/>
+      <c r="J42" s="140"/>
+      <c r="K42" s="141"/>
       <c r="L42" s="49"/>
       <c r="O42" s="127">
         <v>20.60000000000003</v>
@@ -5398,19 +5485,19 @@
       <c r="AT42" s="21"/>
     </row>
     <row r="43" spans="1:46" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="198" t="s">
+      <c r="A43" s="144" t="s">
         <v>68</v>
       </c>
-      <c r="B43" s="162"/>
-      <c r="C43" s="162"/>
-      <c r="D43" s="162"/>
-      <c r="E43" s="162"/>
-      <c r="F43" s="162"/>
-      <c r="G43" s="162"/>
-      <c r="H43" s="162"/>
-      <c r="I43" s="162"/>
-      <c r="J43" s="162"/>
-      <c r="K43" s="138"/>
+      <c r="B43" s="145"/>
+      <c r="C43" s="145"/>
+      <c r="D43" s="145"/>
+      <c r="E43" s="145"/>
+      <c r="F43" s="145"/>
+      <c r="G43" s="145"/>
+      <c r="H43" s="145"/>
+      <c r="I43" s="145"/>
+      <c r="J43" s="145"/>
+      <c r="K43" s="146"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
@@ -5526,10 +5613,10 @@
     <row r="45" spans="1:46" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="3"/>
       <c r="B45" s="63"/>
-      <c r="C45" s="199" t="s">
+      <c r="C45" s="147" t="s">
         <v>69</v>
       </c>
-      <c r="D45" s="160"/>
+      <c r="D45" s="143"/>
       <c r="E45" s="63"/>
       <c r="F45" s="64" t="s">
         <v>70</v>
@@ -5592,8 +5679,8 @@
     <row r="46" spans="1:46" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="20"/>
       <c r="B46" s="20"/>
-      <c r="C46" s="160"/>
-      <c r="D46" s="160"/>
+      <c r="C46" s="143"/>
+      <c r="D46" s="143"/>
       <c r="E46" s="65"/>
       <c r="F46" s="20"/>
       <c r="G46" s="20"/>
@@ -5650,8 +5737,8 @@
     <row r="47" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="20"/>
       <c r="B47" s="20"/>
-      <c r="C47" s="160"/>
-      <c r="D47" s="160"/>
+      <c r="C47" s="143"/>
+      <c r="D47" s="143"/>
       <c r="E47" s="20"/>
       <c r="F47" s="20" t="s">
         <v>54</v>
@@ -5716,8 +5803,8 @@
     <row r="48" spans="1:46" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="20"/>
       <c r="B48" s="20"/>
-      <c r="C48" s="160"/>
-      <c r="D48" s="160"/>
+      <c r="C48" s="143"/>
+      <c r="D48" s="143"/>
       <c r="E48" s="3"/>
       <c r="F48" s="50" t="str">
         <f>+IF(G20="","",(G20*G24)/(G21+G20-G22))</f>
@@ -5780,8 +5867,8 @@
     <row r="49" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="20"/>
       <c r="B49" s="20"/>
-      <c r="C49" s="160"/>
-      <c r="D49" s="160"/>
+      <c r="C49" s="143"/>
+      <c r="D49" s="143"/>
       <c r="E49" s="20"/>
       <c r="F49" s="54" t="e">
         <f>1/((D32/(100*F54))+(F32/(100*F48)))</f>
@@ -5841,8 +5928,8 @@
     <row r="50" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="20"/>
       <c r="B50" s="20"/>
-      <c r="C50" s="160"/>
-      <c r="D50" s="160"/>
+      <c r="C50" s="143"/>
+      <c r="D50" s="143"/>
       <c r="E50" s="20"/>
       <c r="F50" s="56" t="e">
         <f>F48*G48</f>
@@ -6093,12 +6180,12 @@
         <f>F51/(F51-F52)</f>
         <v>1.5789473684210527</v>
       </c>
-      <c r="G54" s="197" t="s">
+      <c r="G54" s="142" t="s">
         <v>67</v>
       </c>
-      <c r="H54" s="160"/>
-      <c r="I54" s="160"/>
-      <c r="J54" s="160"/>
+      <c r="H54" s="143"/>
+      <c r="I54" s="143"/>
+      <c r="J54" s="143"/>
       <c r="K54" s="20"/>
       <c r="L54" s="20"/>
       <c r="M54" s="20"/>
@@ -53209,51 +53296,6 @@
     </row>
   </sheetData>
   <mergeCells count="61">
-    <mergeCell ref="O18:Y19"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="R20:S20"/>
-    <mergeCell ref="U20:V20"/>
-    <mergeCell ref="X20:Y20"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="G54:J54"/>
-    <mergeCell ref="A43:K43"/>
-    <mergeCell ref="C45:D50"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="A37:E42"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="A36:E36"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C30:G30"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C33:D34"/>
-    <mergeCell ref="E33:G34"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="B11:J11"/>
-    <mergeCell ref="C13:K13"/>
-    <mergeCell ref="AO1:AQ1"/>
-    <mergeCell ref="C2:H4"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="AG3:AJ5"/>
-    <mergeCell ref="B5:J5"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="I4:K4"/>
     <mergeCell ref="I36:K36"/>
     <mergeCell ref="A1:B4"/>
     <mergeCell ref="C1:H1"/>
@@ -53270,6 +53312,51 @@
     <mergeCell ref="C7:F7"/>
     <mergeCell ref="C8:F8"/>
     <mergeCell ref="G8:H8"/>
+    <mergeCell ref="AO1:AQ1"/>
+    <mergeCell ref="C2:H4"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="AG3:AJ5"/>
+    <mergeCell ref="B5:J5"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="B11:J11"/>
+    <mergeCell ref="C13:K13"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C33:D34"/>
+    <mergeCell ref="E33:G34"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C30:G30"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="G54:J54"/>
+    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="C45:D50"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="A37:E42"/>
+    <mergeCell ref="O18:Y19"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="U20:V20"/>
+    <mergeCell ref="X20:Y20"/>
   </mergeCells>
   <conditionalFormatting sqref="C12:D12 C32:D32 F32">
     <cfRule type="containsBlanks" dxfId="6" priority="2">
@@ -53346,11 +53433,11 @@
       <c r="E3" s="89"/>
     </row>
     <row r="4" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C4" s="205" t="s">
+      <c r="C4" s="209" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="206"/>
-      <c r="E4" s="206"/>
+      <c r="D4" s="210"/>
+      <c r="E4" s="210"/>
     </row>
     <row r="5" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C5" s="90" t="s">

</xml_diff>